<commit_message>
Fix Class 5 syllabus Excel to use NCERT chapter names and improve re-upload preview.
Chapter Name now matches the textbook; mentor head goes in Remarks. File input resets so the same file can be previewed again.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/samples/syllabus-import/CBSE_Class5_Maths_Syllabus_2026-27.xlsx
+++ b/public/samples/syllabus-import/CBSE_Class5_Maths_Syllabus_2026-27.xlsx
@@ -38,10 +38,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Number System</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> We the Travellers—I</t>
+    <t>We the Travellers—I</t>
   </si>
   <si>
     <t>Large Numbers in Travel</t>
@@ -50,7 +47,7 @@
     <t>Reading and writing numbers up to lakhs in journey contexts</t>
   </si>
   <si>
-    <t>NCERT opening chapter</t>
+    <t>Head: Number System · NCERT opening chapter</t>
   </si>
   <si>
     <t>Routes and Distances</t>
@@ -59,16 +56,16 @@
     <t>Interpreting route charts, comparing distances between places</t>
   </si>
   <si>
+    <t>Head: Number System</t>
+  </si>
+  <si>
     <t>Planning a Journey</t>
   </si>
   <si>
     <t>Estimating cost, time and resources for a trip</t>
   </si>
   <si>
-    <t>Ratio &amp; Proportion</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Fractions</t>
+    <t>Fractions</t>
   </si>
   <si>
     <t>Unit and Like Fractions</t>
@@ -77,6 +74,9 @@
     <t>Understanding numerator, denominator and equal parts of a whole</t>
   </si>
   <si>
+    <t>Head: Ratio &amp; Proportion</t>
+  </si>
+  <si>
     <t>Equivalent Fractions</t>
   </si>
   <si>
@@ -89,10 +89,7 @@
     <t>Ordering fractions with same denominator or using benchmarks</t>
   </si>
   <si>
-    <t>Geometry</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Angles as Turns</t>
+    <t>Angles as Turns</t>
   </si>
   <si>
     <t>Turns as Fractions of a Circle</t>
@@ -101,6 +98,9 @@
     <t>Full, half, quarter and three-quarter turns</t>
   </si>
   <si>
+    <t>Head: Geometry</t>
+  </si>
+  <si>
     <t>Measuring Turns</t>
   </si>
   <si>
@@ -113,10 +113,7 @@
     <t>Describing direction change using turn language</t>
   </si>
   <si>
-    <t>Speed Distance Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> We the Travellers—II</t>
+    <t>We the Travellers—II</t>
   </si>
   <si>
     <t>Reading Timetables</t>
@@ -125,6 +122,9 @@
     <t>Using bus and train schedules to plan travel</t>
   </si>
   <si>
+    <t>Head: Speed Distance Time</t>
+  </si>
+  <si>
     <t>Distance and Time Estimates</t>
   </si>
   <si>
@@ -137,10 +137,7 @@
     <t>Addition and subtraction in route-planning contexts</t>
   </si>
   <si>
-    <t>Perimeter and Area</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Far and Near</t>
+    <t>Far and Near</t>
   </si>
   <si>
     <t>Comparing Distances</t>
@@ -149,6 +146,9 @@
     <t>Near/far, longer/shorter using non-standard units</t>
   </si>
   <si>
+    <t>Head: Perimeter and Area</t>
+  </si>
+  <si>
     <t>Standard Units of Length</t>
   </si>
   <si>
@@ -161,7 +161,7 @@
     <t>Addition and subtraction problems involving distance</t>
   </si>
   <si>
-    <t xml:space="preserve"> The Dairy Farm</t>
+    <t>The Dairy Farm</t>
   </si>
   <si>
     <t>Multiplication in Farming</t>
@@ -182,7 +182,7 @@
     <t>Simple cost and quantity problems in a dairy setting</t>
   </si>
   <si>
-    <t xml:space="preserve"> Shapes and Patterns</t>
+    <t>Shapes and Patterns</t>
   </si>
   <si>
     <t>2D Shapes and Properties</t>
@@ -203,7 +203,7 @@
     <t>Designing borders, rangoli and repeating motifs</t>
   </si>
   <si>
-    <t xml:space="preserve"> Weight and Capacity</t>
+    <t>Weight and Capacity</t>
   </si>
   <si>
     <t>Kilograms and Grams</t>
@@ -224,7 +224,7 @@
     <t>Applied problems on shopping and cooking quantities</t>
   </si>
   <si>
-    <t xml:space="preserve"> Coconut Farm</t>
+    <t>Coconut Farm</t>
   </si>
   <si>
     <t>Fractions of a Harvest</t>
@@ -245,7 +245,7 @@
     <t>Simple profit and sharing problems using fractions</t>
   </si>
   <si>
-    <t xml:space="preserve"> Symmetrical Designs</t>
+    <t>Symmetrical Designs</t>
   </si>
   <si>
     <t>Line Symmetry</t>
@@ -266,7 +266,7 @@
     <t>Creating symmetric rangoli, kolam and craft designs</t>
   </si>
   <si>
-    <t xml:space="preserve"> Grandmother's Quilt</t>
+    <t>Grandmother's Quilt</t>
   </si>
   <si>
     <t>Patchwork Patterns</t>
@@ -287,7 +287,7 @@
     <t>Planning rows, columns and repeating colour blocks</t>
   </si>
   <si>
-    <t xml:space="preserve"> Racing Seconds</t>
+    <t>Racing Seconds</t>
   </si>
   <si>
     <t>Reading Time to the Second</t>
@@ -308,7 +308,7 @@
     <t>Calculating time taken in short-duration events</t>
   </si>
   <si>
-    <t xml:space="preserve"> Animal Jumps</t>
+    <t>Animal Jumps</t>
   </si>
   <si>
     <t>Measuring Jump Lengths</t>
@@ -329,7 +329,7 @@
     <t>Finding a typical jump length from a small data set</t>
   </si>
   <si>
-    <t xml:space="preserve"> Maps and Locations</t>
+    <t>Maps and Locations</t>
   </si>
   <si>
     <t>Grid References</t>
@@ -350,16 +350,16 @@
     <t>Simple scale reading (e.g. 1 cm = 1 km)</t>
   </si>
   <si>
-    <t>Statistics</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Data Through Pictures</t>
+    <t>Data Through Pictures</t>
   </si>
   <si>
     <t>Collecting and Tallying Data</t>
   </si>
   <si>
     <t>Recording observations using tally marks</t>
+  </si>
+  <si>
+    <t>Head: Statistics</t>
   </si>
   <si>
     <t>Pictographs</t>
@@ -715,12 +715,12 @@
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="25.851" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="10.569" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="36.42" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="75.41" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="25.851" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="51.845" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -753,20 +753,17 @@
       <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
         <v>10</v>
-      </c>
-      <c r="F2">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -776,17 +773,17 @@
       <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
       <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3" t="s">
         <v>13</v>
-      </c>
-      <c r="F3">
-        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -796,9 +793,6 @@
       <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
       <c r="D4" t="s">
         <v>14</v>
       </c>
@@ -807,6 +801,9 @@
       </c>
       <c r="F4">
         <v>3</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -816,17 +813,17 @@
       <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>18</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5" t="s">
         <v>19</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -836,9 +833,6 @@
       <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
       <c r="D6" t="s">
         <v>20</v>
       </c>
@@ -847,6 +841,9 @@
       </c>
       <c r="F6">
         <v>4</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -856,9 +853,6 @@
       <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
       <c r="D7" t="s">
         <v>22</v>
       </c>
@@ -868,6 +862,9 @@
       <c r="F7">
         <v>3</v>
       </c>
+      <c r="G7" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8">
@@ -876,17 +873,17 @@
       <c r="B8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>25</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>26</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8">
+        <v>3</v>
+      </c>
+      <c r="G8" t="s">
         <v>27</v>
-      </c>
-      <c r="F8">
-        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -896,9 +893,6 @@
       <c r="B9" t="s">
         <v>24</v>
       </c>
-      <c r="C9" t="s">
-        <v>25</v>
-      </c>
       <c r="D9" t="s">
         <v>28</v>
       </c>
@@ -908,6 +902,9 @@
       <c r="F9">
         <v>3</v>
       </c>
+      <c r="G9" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10">
@@ -916,9 +913,6 @@
       <c r="B10" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
       <c r="D10" t="s">
         <v>30</v>
       </c>
@@ -928,6 +922,9 @@
       <c r="F10">
         <v>2</v>
       </c>
+      <c r="G10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11">
@@ -936,17 +933,17 @@
       <c r="B11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>33</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>34</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11" t="s">
         <v>35</v>
-      </c>
-      <c r="F11">
-        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -956,9 +953,6 @@
       <c r="B12" t="s">
         <v>32</v>
       </c>
-      <c r="C12" t="s">
-        <v>33</v>
-      </c>
       <c r="D12" t="s">
         <v>36</v>
       </c>
@@ -968,6 +962,9 @@
       <c r="F12">
         <v>4</v>
       </c>
+      <c r="G12" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13">
@@ -976,9 +973,6 @@
       <c r="B13" t="s">
         <v>32</v>
       </c>
-      <c r="C13" t="s">
-        <v>33</v>
-      </c>
       <c r="D13" t="s">
         <v>38</v>
       </c>
@@ -987,6 +981,9 @@
       </c>
       <c r="F13">
         <v>3</v>
+      </c>
+      <c r="G13" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -996,17 +993,17 @@
       <c r="B14" t="s">
         <v>40</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>41</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>42</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14" t="s">
         <v>43</v>
-      </c>
-      <c r="F14">
-        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1016,9 +1013,6 @@
       <c r="B15" t="s">
         <v>40</v>
       </c>
-      <c r="C15" t="s">
-        <v>41</v>
-      </c>
       <c r="D15" t="s">
         <v>44</v>
       </c>
@@ -1027,6 +1021,9 @@
       </c>
       <c r="F15">
         <v>4</v>
+      </c>
+      <c r="G15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1036,9 +1033,6 @@
       <c r="B16" t="s">
         <v>40</v>
       </c>
-      <c r="C16" t="s">
-        <v>41</v>
-      </c>
       <c r="D16" t="s">
         <v>46</v>
       </c>
@@ -1047,6 +1041,9 @@
       </c>
       <c r="F16">
         <v>3</v>
+      </c>
+      <c r="G16" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1054,9 +1051,6 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" t="s">
         <v>48</v>
       </c>
       <c r="D17" t="s">
@@ -1067,6 +1061,9 @@
       </c>
       <c r="F17">
         <v>4</v>
+      </c>
+      <c r="G17" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1074,9 +1071,6 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" t="s">
         <v>48</v>
       </c>
       <c r="D18" t="s">
@@ -1087,6 +1081,9 @@
       </c>
       <c r="F18">
         <v>4</v>
+      </c>
+      <c r="G18" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1094,9 +1091,6 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" t="s">
         <v>48</v>
       </c>
       <c r="D19" t="s">
@@ -1107,6 +1101,9 @@
       </c>
       <c r="F19">
         <v>3</v>
+      </c>
+      <c r="G19" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1114,9 +1111,6 @@
         <v>7</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" t="s">
         <v>55</v>
       </c>
       <c r="D20" t="s">
@@ -1127,6 +1121,9 @@
       </c>
       <c r="F20">
         <v>3</v>
+      </c>
+      <c r="G20" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1134,9 +1131,6 @@
         <v>7</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" t="s">
         <v>55</v>
       </c>
       <c r="D21" t="s">
@@ -1147,6 +1141,9 @@
       </c>
       <c r="F21">
         <v>3</v>
+      </c>
+      <c r="G21" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1154,9 +1151,6 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" t="s">
         <v>55</v>
       </c>
       <c r="D22" t="s">
@@ -1167,6 +1161,9 @@
       </c>
       <c r="F22">
         <v>2</v>
+      </c>
+      <c r="G22" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1174,9 +1171,6 @@
         <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" t="s">
         <v>62</v>
       </c>
       <c r="D23" t="s">
@@ -1187,6 +1181,9 @@
       </c>
       <c r="F23">
         <v>4</v>
+      </c>
+      <c r="G23" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1194,9 +1191,6 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" t="s">
         <v>62</v>
       </c>
       <c r="D24" t="s">
@@ -1207,6 +1201,9 @@
       </c>
       <c r="F24">
         <v>4</v>
+      </c>
+      <c r="G24" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1214,9 +1211,6 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" t="s">
         <v>62</v>
       </c>
       <c r="D25" t="s">
@@ -1227,6 +1221,9 @@
       </c>
       <c r="F25">
         <v>3</v>
+      </c>
+      <c r="G25" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1234,9 +1231,6 @@
         <v>9</v>
       </c>
       <c r="B26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" t="s">
         <v>69</v>
       </c>
       <c r="D26" t="s">
@@ -1247,6 +1241,9 @@
       </c>
       <c r="F26">
         <v>4</v>
+      </c>
+      <c r="G26" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1254,9 +1251,6 @@
         <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" t="s">
         <v>69</v>
       </c>
       <c r="D27" t="s">
@@ -1267,6 +1261,9 @@
       </c>
       <c r="F27">
         <v>3</v>
+      </c>
+      <c r="G27" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1274,9 +1271,6 @@
         <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>16</v>
-      </c>
-      <c r="C28" t="s">
         <v>69</v>
       </c>
       <c r="D28" t="s">
@@ -1287,6 +1281,9 @@
       </c>
       <c r="F28">
         <v>3</v>
+      </c>
+      <c r="G28" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1294,9 +1291,6 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>24</v>
-      </c>
-      <c r="C29" t="s">
         <v>76</v>
       </c>
       <c r="D29" t="s">
@@ -1307,6 +1301,9 @@
       </c>
       <c r="F29">
         <v>3</v>
+      </c>
+      <c r="G29" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1314,9 +1311,6 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>24</v>
-      </c>
-      <c r="C30" t="s">
         <v>76</v>
       </c>
       <c r="D30" t="s">
@@ -1327,6 +1321,9 @@
       </c>
       <c r="F30">
         <v>3</v>
+      </c>
+      <c r="G30" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1334,9 +1331,6 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C31" t="s">
         <v>76</v>
       </c>
       <c r="D31" t="s">
@@ -1347,6 +1341,9 @@
       </c>
       <c r="F31">
         <v>2</v>
+      </c>
+      <c r="G31" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1354,9 +1351,6 @@
         <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C32" t="s">
         <v>83</v>
       </c>
       <c r="D32" t="s">
@@ -1367,6 +1361,9 @@
       </c>
       <c r="F32">
         <v>3</v>
+      </c>
+      <c r="G32" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1374,9 +1371,6 @@
         <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>24</v>
-      </c>
-      <c r="C33" t="s">
         <v>83</v>
       </c>
       <c r="D33" t="s">
@@ -1387,6 +1381,9 @@
       </c>
       <c r="F33">
         <v>3</v>
+      </c>
+      <c r="G33" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1394,9 +1391,6 @@
         <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>24</v>
-      </c>
-      <c r="C34" t="s">
         <v>83</v>
       </c>
       <c r="D34" t="s">
@@ -1407,6 +1401,9 @@
       </c>
       <c r="F34">
         <v>2</v>
+      </c>
+      <c r="G34" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1414,9 +1411,6 @@
         <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" t="s">
         <v>90</v>
       </c>
       <c r="D35" t="s">
@@ -1427,6 +1421,9 @@
       </c>
       <c r="F35">
         <v>3</v>
+      </c>
+      <c r="G35" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1434,9 +1431,6 @@
         <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
-      </c>
-      <c r="C36" t="s">
         <v>90</v>
       </c>
       <c r="D36" t="s">
@@ -1447,6 +1441,9 @@
       </c>
       <c r="F36">
         <v>4</v>
+      </c>
+      <c r="G36" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1454,9 +1451,6 @@
         <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" t="s">
         <v>90</v>
       </c>
       <c r="D37" t="s">
@@ -1467,6 +1461,9 @@
       </c>
       <c r="F37">
         <v>3</v>
+      </c>
+      <c r="G37" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -1474,9 +1471,6 @@
         <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>40</v>
-      </c>
-      <c r="C38" t="s">
         <v>97</v>
       </c>
       <c r="D38" t="s">
@@ -1487,6 +1481,9 @@
       </c>
       <c r="F38">
         <v>3</v>
+      </c>
+      <c r="G38" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -1494,9 +1491,6 @@
         <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
-      </c>
-      <c r="C39" t="s">
         <v>97</v>
       </c>
       <c r="D39" t="s">
@@ -1507,6 +1501,9 @@
       </c>
       <c r="F39">
         <v>3</v>
+      </c>
+      <c r="G39" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -1514,9 +1511,6 @@
         <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
-      </c>
-      <c r="C40" t="s">
         <v>97</v>
       </c>
       <c r="D40" t="s">
@@ -1527,6 +1521,9 @@
       </c>
       <c r="F40">
         <v>3</v>
+      </c>
+      <c r="G40" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -1534,9 +1531,6 @@
         <v>14</v>
       </c>
       <c r="B41" t="s">
-        <v>24</v>
-      </c>
-      <c r="C41" t="s">
         <v>104</v>
       </c>
       <c r="D41" t="s">
@@ -1547,6 +1541,9 @@
       </c>
       <c r="F41">
         <v>4</v>
+      </c>
+      <c r="G41" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -1554,9 +1551,6 @@
         <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>24</v>
-      </c>
-      <c r="C42" t="s">
         <v>104</v>
       </c>
       <c r="D42" t="s">
@@ -1567,6 +1561,9 @@
       </c>
       <c r="F42">
         <v>3</v>
+      </c>
+      <c r="G42" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -1574,9 +1571,6 @@
         <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>24</v>
-      </c>
-      <c r="C43" t="s">
         <v>104</v>
       </c>
       <c r="D43" t="s">
@@ -1587,6 +1581,9 @@
       </c>
       <c r="F43">
         <v>4</v>
+      </c>
+      <c r="G43" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1596,17 +1593,17 @@
       <c r="B44" t="s">
         <v>111</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>112</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>113</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44" t="s">
         <v>114</v>
-      </c>
-      <c r="F44">
-        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -1616,9 +1613,6 @@
       <c r="B45" t="s">
         <v>111</v>
       </c>
-      <c r="C45" t="s">
-        <v>112</v>
-      </c>
       <c r="D45" t="s">
         <v>115</v>
       </c>
@@ -1627,6 +1621,9 @@
       </c>
       <c r="F45">
         <v>4</v>
+      </c>
+      <c r="G45" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -1636,9 +1633,6 @@
       <c r="B46" t="s">
         <v>111</v>
       </c>
-      <c r="C46" t="s">
-        <v>112</v>
-      </c>
       <c r="D46" t="s">
         <v>117</v>
       </c>
@@ -1647,6 +1641,9 @@
       </c>
       <c r="F46">
         <v>3</v>
+      </c>
+      <c r="G46" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Map Class 5 chapter column to Chapter Head on syllabus Excel import.
FINAL 5.xlsx uses chapter for mentor heads (Number System, Geometry); import now sets chapter_head_id and auto-creates missing heads on save.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/samples/syllabus-import/CBSE_Class5_Maths_Syllabus_2026-27.xlsx
+++ b/public/samples/syllabus-import/CBSE_Class5_Maths_Syllabus_2026-27.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="117">
   <si>
     <t>Chapter No.</t>
   </si>
@@ -35,30 +35,24 @@
     <t>Approx. Periods</t>
   </si>
   <si>
-    <t>Remarks</t>
-  </si>
-  <si>
     <t>We the Travellers—I</t>
   </si>
   <si>
+    <t>Number System</t>
+  </si>
+  <si>
     <t>Large Numbers in Travel</t>
   </si>
   <si>
     <t>Reading and writing numbers up to lakhs in journey contexts</t>
   </si>
   <si>
-    <t>Head: Number System · NCERT opening chapter</t>
-  </si>
-  <si>
     <t>Routes and Distances</t>
   </si>
   <si>
     <t>Interpreting route charts, comparing distances between places</t>
   </si>
   <si>
-    <t>Head: Number System</t>
-  </si>
-  <si>
     <t>Planning a Journey</t>
   </si>
   <si>
@@ -68,15 +62,15 @@
     <t>Fractions</t>
   </si>
   <si>
+    <t>Ratio &amp; Proportion</t>
+  </si>
+  <si>
     <t>Unit and Like Fractions</t>
   </si>
   <si>
     <t>Understanding numerator, denominator and equal parts of a whole</t>
   </si>
   <si>
-    <t>Head: Ratio &amp; Proportion</t>
-  </si>
-  <si>
     <t>Equivalent Fractions</t>
   </si>
   <si>
@@ -92,15 +86,15 @@
     <t>Angles as Turns</t>
   </si>
   <si>
+    <t>Geometry</t>
+  </si>
+  <si>
     <t>Turns as Fractions of a Circle</t>
   </si>
   <si>
     <t>Full, half, quarter and three-quarter turns</t>
   </si>
   <si>
-    <t>Head: Geometry</t>
-  </si>
-  <si>
     <t>Measuring Turns</t>
   </si>
   <si>
@@ -116,15 +110,15 @@
     <t>We the Travellers—II</t>
   </si>
   <si>
+    <t>Speed Distance Time</t>
+  </si>
+  <si>
     <t>Reading Timetables</t>
   </si>
   <si>
     <t>Using bus and train schedules to plan travel</t>
   </si>
   <si>
-    <t>Head: Speed Distance Time</t>
-  </si>
-  <si>
     <t>Distance and Time Estimates</t>
   </si>
   <si>
@@ -140,15 +134,15 @@
     <t>Far and Near</t>
   </si>
   <si>
+    <t>Perimeter and Area</t>
+  </si>
+  <si>
     <t>Comparing Distances</t>
   </si>
   <si>
     <t>Near/far, longer/shorter using non-standard units</t>
   </si>
   <si>
-    <t>Head: Perimeter and Area</t>
-  </si>
-  <si>
     <t>Standard Units of Length</t>
   </si>
   <si>
@@ -353,13 +347,13 @@
     <t>Data Through Pictures</t>
   </si>
   <si>
+    <t>Statistics</t>
+  </si>
+  <si>
     <t>Collecting and Tallying Data</t>
   </si>
   <si>
     <t>Recording observations using tally marks</t>
-  </si>
-  <si>
-    <t>Head: Statistics</t>
   </si>
   <si>
     <t>Pictographs</t>
@@ -716,11 +710,10 @@
   <cols>
     <col min="1" max="1" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="10.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="23.423" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="36.42" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="75.41" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="51.845" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -742,15 +735,15 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" t="s">
@@ -761,9 +754,6 @@
       </c>
       <c r="F2">
         <v>4</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -771,19 +761,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
       <c r="F3">
         <v>3</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -791,19 +781,19 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F4">
         <v>3</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -811,19 +801,19 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" t="s">
-        <v>18</v>
-      </c>
       <c r="F5">
         <v>4</v>
-      </c>
-      <c r="G5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -831,19 +821,19 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F6">
         <v>4</v>
-      </c>
-      <c r="G6" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -851,19 +841,19 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F7">
         <v>3</v>
-      </c>
-      <c r="G7" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -871,19 +861,19 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
         <v>24</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>25</v>
       </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
       <c r="F8">
         <v>3</v>
-      </c>
-      <c r="G8" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -891,19 +881,19 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F9">
         <v>3</v>
-      </c>
-      <c r="G9" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -911,39 +901,39 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F10">
         <v>2</v>
       </c>
-      <c r="G10" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11">
         <v>4</v>
       </c>
       <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
         <v>32</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>33</v>
       </c>
-      <c r="E11" t="s">
-        <v>34</v>
-      </c>
       <c r="F11">
         <v>4</v>
-      </c>
-      <c r="G11" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -951,19 +941,19 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F12">
         <v>4</v>
-      </c>
-      <c r="G12" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -971,19 +961,19 @@
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F13">
         <v>3</v>
-      </c>
-      <c r="G13" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -991,19 +981,19 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" t="s">
         <v>40</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>41</v>
       </c>
-      <c r="E14" t="s">
-        <v>42</v>
-      </c>
       <c r="F14">
         <v>3</v>
-      </c>
-      <c r="G14" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1011,19 +1001,19 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>38</v>
+      </c>
+      <c r="C15" t="s">
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E15" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F15">
         <v>4</v>
-      </c>
-      <c r="G15" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1031,19 +1021,19 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>38</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F16">
         <v>3</v>
-      </c>
-      <c r="G16" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1051,19 +1041,19 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" t="s">
         <v>48</v>
       </c>
-      <c r="D17" t="s">
-        <v>49</v>
-      </c>
-      <c r="E17" t="s">
-        <v>50</v>
-      </c>
       <c r="F17">
         <v>4</v>
-      </c>
-      <c r="G17" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1071,19 +1061,19 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="C18" t="s">
+        <v>7</v>
       </c>
       <c r="D18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F18">
         <v>4</v>
-      </c>
-      <c r="G18" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1091,19 +1081,19 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F19">
         <v>3</v>
-      </c>
-      <c r="G19" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1111,19 +1101,19 @@
         <v>7</v>
       </c>
       <c r="B20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" t="s">
         <v>55</v>
       </c>
-      <c r="D20" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" t="s">
-        <v>57</v>
-      </c>
       <c r="F20">
         <v>3</v>
-      </c>
-      <c r="G20" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1131,19 +1121,19 @@
         <v>7</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>53</v>
+      </c>
+      <c r="C21" t="s">
+        <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F21">
         <v>3</v>
-      </c>
-      <c r="G21" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1151,19 +1141,19 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>53</v>
+      </c>
+      <c r="C22" t="s">
+        <v>23</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F22">
         <v>2</v>
-      </c>
-      <c r="G22" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1171,19 +1161,19 @@
         <v>8</v>
       </c>
       <c r="B23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" t="s">
+        <v>61</v>
+      </c>
+      <c r="E23" t="s">
         <v>62</v>
       </c>
-      <c r="D23" t="s">
-        <v>63</v>
-      </c>
-      <c r="E23" t="s">
-        <v>64</v>
-      </c>
       <c r="F23">
         <v>4</v>
-      </c>
-      <c r="G23" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1191,19 +1181,19 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>62</v>
+        <v>60</v>
+      </c>
+      <c r="C24" t="s">
+        <v>39</v>
       </c>
       <c r="D24" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F24">
         <v>4</v>
-      </c>
-      <c r="G24" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1211,19 +1201,19 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>62</v>
+        <v>60</v>
+      </c>
+      <c r="C25" t="s">
+        <v>39</v>
       </c>
       <c r="D25" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E25" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F25">
         <v>3</v>
-      </c>
-      <c r="G25" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1231,19 +1221,19 @@
         <v>9</v>
       </c>
       <c r="B26" t="s">
+        <v>67</v>
+      </c>
+      <c r="C26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" t="s">
+        <v>68</v>
+      </c>
+      <c r="E26" t="s">
         <v>69</v>
       </c>
-      <c r="D26" t="s">
-        <v>70</v>
-      </c>
-      <c r="E26" t="s">
-        <v>71</v>
-      </c>
       <c r="F26">
         <v>4</v>
-      </c>
-      <c r="G26" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1251,19 +1241,19 @@
         <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>67</v>
+      </c>
+      <c r="C27" t="s">
+        <v>15</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E27" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F27">
         <v>3</v>
-      </c>
-      <c r="G27" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1271,19 +1261,19 @@
         <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>69</v>
+        <v>67</v>
+      </c>
+      <c r="C28" t="s">
+        <v>15</v>
       </c>
       <c r="D28" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F28">
         <v>3</v>
-      </c>
-      <c r="G28" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1291,19 +1281,19 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" t="s">
+        <v>75</v>
+      </c>
+      <c r="E29" t="s">
         <v>76</v>
       </c>
-      <c r="D29" t="s">
-        <v>77</v>
-      </c>
-      <c r="E29" t="s">
-        <v>78</v>
-      </c>
       <c r="F29">
         <v>3</v>
-      </c>
-      <c r="G29" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1311,19 +1301,19 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>74</v>
+      </c>
+      <c r="C30" t="s">
+        <v>23</v>
       </c>
       <c r="D30" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F30">
         <v>3</v>
-      </c>
-      <c r="G30" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1331,19 +1321,19 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>76</v>
+        <v>74</v>
+      </c>
+      <c r="C31" t="s">
+        <v>23</v>
       </c>
       <c r="D31" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E31" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F31">
         <v>2</v>
-      </c>
-      <c r="G31" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1351,19 +1341,19 @@
         <v>11</v>
       </c>
       <c r="B32" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32" t="s">
+        <v>23</v>
+      </c>
+      <c r="D32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E32" t="s">
         <v>83</v>
       </c>
-      <c r="D32" t="s">
-        <v>84</v>
-      </c>
-      <c r="E32" t="s">
-        <v>85</v>
-      </c>
       <c r="F32">
         <v>3</v>
-      </c>
-      <c r="G32" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1371,19 +1361,19 @@
         <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>83</v>
+        <v>81</v>
+      </c>
+      <c r="C33" t="s">
+        <v>23</v>
       </c>
       <c r="D33" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E33" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F33">
         <v>3</v>
-      </c>
-      <c r="G33" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1391,19 +1381,19 @@
         <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>83</v>
+        <v>81</v>
+      </c>
+      <c r="C34" t="s">
+        <v>23</v>
       </c>
       <c r="D34" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E34" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F34">
         <v>2</v>
-      </c>
-      <c r="G34" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1411,19 +1401,19 @@
         <v>12</v>
       </c>
       <c r="B35" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" t="s">
+        <v>31</v>
+      </c>
+      <c r="D35" t="s">
+        <v>89</v>
+      </c>
+      <c r="E35" t="s">
         <v>90</v>
       </c>
-      <c r="D35" t="s">
-        <v>91</v>
-      </c>
-      <c r="E35" t="s">
-        <v>92</v>
-      </c>
       <c r="F35">
         <v>3</v>
-      </c>
-      <c r="G35" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1431,19 +1421,19 @@
         <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>88</v>
+      </c>
+      <c r="C36" t="s">
+        <v>31</v>
       </c>
       <c r="D36" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E36" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F36">
         <v>4</v>
-      </c>
-      <c r="G36" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1451,19 +1441,19 @@
         <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>88</v>
+      </c>
+      <c r="C37" t="s">
+        <v>31</v>
       </c>
       <c r="D37" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E37" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F37">
         <v>3</v>
-      </c>
-      <c r="G37" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -1471,19 +1461,19 @@
         <v>13</v>
       </c>
       <c r="B38" t="s">
+        <v>95</v>
+      </c>
+      <c r="C38" t="s">
+        <v>39</v>
+      </c>
+      <c r="D38" t="s">
+        <v>96</v>
+      </c>
+      <c r="E38" t="s">
         <v>97</v>
       </c>
-      <c r="D38" t="s">
-        <v>98</v>
-      </c>
-      <c r="E38" t="s">
-        <v>99</v>
-      </c>
       <c r="F38">
         <v>3</v>
-      </c>
-      <c r="G38" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -1491,19 +1481,19 @@
         <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>97</v>
+        <v>95</v>
+      </c>
+      <c r="C39" t="s">
+        <v>39</v>
       </c>
       <c r="D39" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E39" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F39">
         <v>3</v>
-      </c>
-      <c r="G39" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -1511,19 +1501,19 @@
         <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>97</v>
+        <v>95</v>
+      </c>
+      <c r="C40" t="s">
+        <v>39</v>
       </c>
       <c r="D40" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E40" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F40">
         <v>3</v>
-      </c>
-      <c r="G40" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -1531,19 +1521,19 @@
         <v>14</v>
       </c>
       <c r="B41" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" t="s">
+        <v>23</v>
+      </c>
+      <c r="D41" t="s">
+        <v>103</v>
+      </c>
+      <c r="E41" t="s">
         <v>104</v>
       </c>
-      <c r="D41" t="s">
-        <v>105</v>
-      </c>
-      <c r="E41" t="s">
-        <v>106</v>
-      </c>
       <c r="F41">
         <v>4</v>
-      </c>
-      <c r="G41" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -1551,19 +1541,19 @@
         <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>104</v>
+        <v>102</v>
+      </c>
+      <c r="C42" t="s">
+        <v>23</v>
       </c>
       <c r="D42" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E42" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F42">
         <v>3</v>
-      </c>
-      <c r="G42" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -1571,19 +1561,19 @@
         <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>104</v>
+        <v>102</v>
+      </c>
+      <c r="C43" t="s">
+        <v>23</v>
       </c>
       <c r="D43" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E43" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F43">
         <v>4</v>
-      </c>
-      <c r="G43" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1591,19 +1581,19 @@
         <v>15</v>
       </c>
       <c r="B44" t="s">
+        <v>109</v>
+      </c>
+      <c r="C44" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" t="s">
         <v>111</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>112</v>
       </c>
-      <c r="E44" t="s">
-        <v>113</v>
-      </c>
       <c r="F44">
         <v>3</v>
-      </c>
-      <c r="G44" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -1611,19 +1601,19 @@
         <v>15</v>
       </c>
       <c r="B45" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="C45" t="s">
+        <v>110</v>
       </c>
       <c r="D45" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E45" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F45">
         <v>4</v>
-      </c>
-      <c r="G45" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -1631,19 +1621,19 @@
         <v>15</v>
       </c>
       <c r="B46" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="C46" t="s">
+        <v>110</v>
       </c>
       <c r="D46" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E46" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F46">
         <v>3</v>
-      </c>
-      <c r="G46" t="s">
-        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>